<commit_message>
Update dormitory guide Excel data
</commit_message>
<xml_diff>
--- a/dormitory_guide_v2.xlsx
+++ b/dormitory_guide_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\0526\dormitory_project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15366760-9461-4050-A489-77D1E03B5F2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{504F95A9-AA92-4709-A911-7C039819D030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="73">
   <si>
     <t>카테고리</t>
   </si>
@@ -240,6 +240,14 @@
   </si>
   <si>
     <t>칼, 도마, 국자, 냄비 등이 있습니다.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>점심메뉴 추천해줘</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>기분이 꿀꿀하다면 꿀꿀 삼겹살!</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -336,7 +344,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -357,6 +365,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -661,7 +675,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1021,6 +1035,17 @@
         <v>70</v>
       </c>
     </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>